<commit_message>
Corrected SL calculation whem multiple MSFName
</commit_message>
<xml_diff>
--- a/Main Input Files/LP MSF mapping.xlsx
+++ b/Main Input Files/LP MSF mapping.xlsx
@@ -5,17 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://riotinto-my.sharepoint.com/personal/oliver_lartigue_riotinto_com/Documents/Documents/31. Tool for LP SL computation/Input Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://riotinto-my.sharepoint.com/personal/oliver_lartigue_riotinto_com/Documents/Documents/31. Tool for LP SL computation/Main Input Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9196A4BE-9526-4D37-A78A-11F0745B5C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{9196A4BE-9526-4D37-A78A-11F0745B5C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C37CD769-5BB4-4459-AFB2-F297CC86E443}"/>
   <bookViews>
-    <workbookView xWindow="13065" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{26E0F985-04E8-41B0-A2C7-BBAD4DDF7EE7}"/>
+    <workbookView xWindow="1872" yWindow="4032" windowWidth="17280" windowHeight="8880" xr2:uid="{26E0F985-04E8-41B0-A2C7-BBAD4DDF7EE7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$179</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1234,6 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7ADCA9-084A-4F6A-B07C-E2482E2DBBC6}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1260,7 +1264,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1502</v>
       </c>
@@ -1280,7 +1284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1502</v>
       </c>
@@ -1300,7 +1304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1320,7 +1324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1340,7 +1344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1360,7 +1364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>3</v>
       </c>
@@ -1380,7 +1384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1618</v>
       </c>
@@ -1400,7 +1404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1618</v>
       </c>
@@ -1420,7 +1424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1440,7 +1444,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1</v>
       </c>
@@ -1460,7 +1464,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1480,7 +1484,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1500,7 +1504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>21</v>
       </c>
@@ -1520,7 +1524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>21</v>
       </c>
@@ -1540,7 +1544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>21</v>
       </c>
@@ -1560,7 +1564,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>21</v>
       </c>
@@ -1580,7 +1584,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>23</v>
       </c>
@@ -1600,7 +1604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>88</v>
       </c>
@@ -1620,7 +1624,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>31</v>
       </c>
@@ -1640,7 +1644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>31</v>
       </c>
@@ -1660,7 +1664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>25</v>
       </c>
@@ -1680,7 +1684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>25</v>
       </c>
@@ -1700,7 +1704,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>25</v>
       </c>
@@ -1720,7 +1724,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
@@ -1740,7 +1744,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1760,7 +1764,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1780,7 +1784,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>25</v>
       </c>
@@ -1800,7 +1804,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>30</v>
       </c>
@@ -1820,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
@@ -1840,7 +1844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>9</v>
       </c>
@@ -1860,7 +1864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>9</v>
       </c>
@@ -1880,7 +1884,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>9</v>
       </c>
@@ -1900,7 +1904,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>9</v>
       </c>
@@ -1920,7 +1924,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>9</v>
       </c>
@@ -1940,7 +1944,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>9</v>
       </c>
@@ -1960,7 +1964,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>9</v>
       </c>
@@ -1980,7 +1984,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>9</v>
       </c>
@@ -2000,7 +2004,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>9</v>
       </c>
@@ -2020,7 +2024,7 @@
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1651</v>
       </c>
@@ -2040,7 +2044,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>87</v>
       </c>
@@ -2060,7 +2064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>46</v>
       </c>
@@ -2080,7 +2084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>46</v>
       </c>
@@ -2100,7 +2104,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>46</v>
       </c>
@@ -2120,7 +2124,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1644</v>
       </c>
@@ -2140,7 +2144,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2160,7 +2164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>49</v>
       </c>
@@ -2180,7 +2184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>49</v>
       </c>
@@ -2200,7 +2204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>50</v>
       </c>
@@ -2220,7 +2224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -2300,7 +2304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>1653</v>
       </c>
@@ -2320,7 +2324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -2340,7 +2344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2360,7 +2364,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>55</v>
       </c>
@@ -2380,7 +2384,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>55</v>
       </c>
@@ -2400,7 +2404,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>55</v>
       </c>
@@ -2420,7 +2424,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>52</v>
       </c>
@@ -2440,7 +2444,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>52</v>
       </c>
@@ -2460,7 +2464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>52</v>
       </c>
@@ -2480,7 +2484,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>52</v>
       </c>
@@ -2500,7 +2504,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>52</v>
       </c>
@@ -2520,7 +2524,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>52</v>
       </c>
@@ -2540,7 +2544,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>60</v>
       </c>
@@ -2560,7 +2564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>60</v>
       </c>
@@ -2580,7 +2584,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>60</v>
       </c>
@@ -2600,7 +2604,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>57</v>
       </c>
@@ -2620,7 +2624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>57</v>
       </c>
@@ -2640,7 +2644,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>57</v>
       </c>
@@ -2660,7 +2664,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>1647</v>
       </c>
@@ -2680,7 +2684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1647</v>
       </c>
@@ -2700,7 +2704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1647</v>
       </c>
@@ -2720,7 +2724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>89</v>
       </c>
@@ -2740,7 +2744,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>65</v>
       </c>
@@ -2760,7 +2764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>65</v>
       </c>
@@ -2780,7 +2784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>65</v>
       </c>
@@ -2800,7 +2804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>64</v>
       </c>
@@ -2820,7 +2824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>64</v>
       </c>
@@ -2840,7 +2844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>64</v>
       </c>
@@ -2860,7 +2864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>67</v>
       </c>
@@ -2880,7 +2884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>68</v>
       </c>
@@ -2900,7 +2904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>86</v>
       </c>
@@ -2920,7 +2924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>83</v>
       </c>
@@ -2940,7 +2944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>83</v>
       </c>
@@ -2960,7 +2964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>83</v>
       </c>
@@ -2980,7 +2984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>83</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>35</v>
       </c>
@@ -3020,7 +3024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>35</v>
       </c>
@@ -3040,7 +3044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>35</v>
       </c>
@@ -3060,7 +3064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>35</v>
       </c>
@@ -3080,7 +3084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>33</v>
       </c>
@@ -3100,7 +3104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>36</v>
       </c>
@@ -3120,7 +3124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>36</v>
       </c>
@@ -3140,7 +3144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>1652</v>
       </c>
@@ -3160,7 +3164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>1642</v>
       </c>
@@ -3180,7 +3184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>1641</v>
       </c>
@@ -3200,7 +3204,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>1643</v>
       </c>
@@ -3220,7 +3224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>39</v>
       </c>
@@ -3240,7 +3244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>38</v>
       </c>
@@ -3260,7 +3264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>38</v>
       </c>
@@ -3280,7 +3284,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>38</v>
       </c>
@@ -3300,7 +3304,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>38</v>
       </c>
@@ -3320,7 +3324,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>38</v>
       </c>
@@ -3340,7 +3344,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>38</v>
       </c>
@@ -3360,7 +3364,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>38</v>
       </c>
@@ -3380,7 +3384,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>40</v>
       </c>
@@ -3400,7 +3404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>41</v>
       </c>
@@ -3420,7 +3424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>41</v>
       </c>
@@ -3440,7 +3444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>42</v>
       </c>
@@ -3460,7 +3464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>42</v>
       </c>
@@ -3480,7 +3484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>42</v>
       </c>
@@ -3500,7 +3504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>42</v>
       </c>
@@ -3520,7 +3524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>42</v>
       </c>
@@ -3540,7 +3544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>42</v>
       </c>
@@ -3560,7 +3564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>42</v>
       </c>
@@ -3580,7 +3584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>43</v>
       </c>
@@ -3600,7 +3604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>43</v>
       </c>
@@ -3620,7 +3624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>1656</v>
       </c>
@@ -3640,7 +3644,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>1657</v>
       </c>
@@ -3660,7 +3664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>84</v>
       </c>
@@ -3680,7 +3684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>84</v>
       </c>
@@ -3700,7 +3704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>71</v>
       </c>
@@ -3720,7 +3724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>71</v>
       </c>
@@ -3740,7 +3744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>72</v>
       </c>
@@ -3760,7 +3764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>72</v>
       </c>
@@ -3780,7 +3784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>72</v>
       </c>
@@ -3800,7 +3804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>72</v>
       </c>
@@ -3820,7 +3824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>70</v>
       </c>
@@ -3840,7 +3844,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>70</v>
       </c>
@@ -3860,7 +3864,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>70</v>
       </c>
@@ -3880,7 +3884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>85</v>
       </c>
@@ -3900,7 +3904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>85</v>
       </c>
@@ -3920,7 +3924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>1645</v>
       </c>
@@ -3940,7 +3944,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>1645</v>
       </c>
@@ -3960,7 +3964,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>1645</v>
       </c>
@@ -3980,7 +3984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>1645</v>
       </c>
@@ -4000,7 +4004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>77</v>
       </c>
@@ -4020,7 +4024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>77</v>
       </c>
@@ -4040,7 +4044,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>77</v>
       </c>
@@ -4060,7 +4064,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>77</v>
       </c>
@@ -4080,7 +4084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>78</v>
       </c>
@@ -4100,7 +4104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>78</v>
       </c>
@@ -4120,7 +4124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>78</v>
       </c>
@@ -4140,7 +4144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>78</v>
       </c>
@@ -4160,7 +4164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>78</v>
       </c>
@@ -4180,7 +4184,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>78</v>
       </c>
@@ -4200,7 +4204,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>79</v>
       </c>
@@ -4220,7 +4224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>79</v>
       </c>
@@ -4240,7 +4244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>79</v>
       </c>
@@ -4260,7 +4264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>79</v>
       </c>
@@ -4280,7 +4284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>79</v>
       </c>
@@ -4300,7 +4304,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>79</v>
       </c>
@@ -4320,7 +4324,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>79</v>
       </c>
@@ -4340,7 +4344,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>80</v>
       </c>
@@ -4360,7 +4364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>80</v>
       </c>
@@ -4380,7 +4384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>74</v>
       </c>
@@ -4400,7 +4404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>74</v>
       </c>
@@ -4420,7 +4424,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>74</v>
       </c>
@@ -4440,7 +4444,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>74</v>
       </c>
@@ -4460,7 +4464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>75</v>
       </c>
@@ -4480,7 +4484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>75</v>
       </c>
@@ -4500,7 +4504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>75</v>
       </c>
@@ -4520,7 +4524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>75</v>
       </c>
@@ -4540,7 +4544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>75</v>
       </c>
@@ -4560,7 +4564,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>75</v>
       </c>
@@ -4580,7 +4584,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>76</v>
       </c>
@@ -4600,7 +4604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>76</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>76</v>
       </c>
@@ -4640,7 +4644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>76</v>
       </c>
@@ -4660,7 +4664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>76</v>
       </c>
@@ -4680,7 +4684,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>76</v>
       </c>
@@ -4700,7 +4704,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>76</v>
       </c>
@@ -4720,7 +4724,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>82</v>
       </c>
@@ -4740,7 +4744,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>82</v>
       </c>
@@ -4760,7 +4764,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>82</v>
       </c>
@@ -4780,7 +4784,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>82</v>
       </c>
@@ -4800,7 +4804,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>82</v>
       </c>
@@ -4821,6 +4825,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F179" xr:uid="{AF7ADCA9-084A-4F6A-B07C-E2482E2DBBC6}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="HD Plant"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>